<commit_message>
Added Daria and Eoin
</commit_message>
<xml_diff>
--- a/Noir Wingman/Assets/Sheets/Demo Dialogue/Eoin Richardson/Rookie_Draft_1.xlsx
+++ b/Noir Wingman/Assets/Sheets/Demo Dialogue/Eoin Richardson/Rookie_Draft_1.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b685ca5cabcdd482/Desktop/NoirWingman/Noir Wingman/Assets/Sheets/Demo Dialogue/Eoin Richardson/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="148" documentId="8_{26725DD3-B018-4E80-AFB8-797A6CF7C32F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{101ED1AE-8893-4F9E-A721-52A39F82F6AD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{325FF245-919F-4DE7-984C-269CEA87FA4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{A85544C4-B6D9-419A-8FBF-C64C862E95D0}"/>
   </bookViews>
   <sheets>
-    <sheet name="Rookie_Intro_1" sheetId="1" r:id="rId1"/>
+    <sheet name="Rookie_Draft_1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="71">
   <si>
     <t>Reaction</t>
   </si>
@@ -89,15 +89,9 @@
     <t>Why Here?</t>
   </si>
   <si>
-    <t>What brings you here? Doesn’t really seem like your scene.</t>
-  </si>
-  <si>
     <t>Sad|Angry|Sad</t>
   </si>
   <si>
-    <t>Uh- well- y’know, the boys were going out, and they ended up inviting me along. I didn’t know we were going- to be honest, I assumed we were going to go get dinner down at the diner or something, but- uh- I guess not. I tried to leave, but I saw Sam, and I just… didn’t want to leave the guy alone, y’know?|*He stares pointedly at me, the resentment writ large on his face.|I do. Trust me.</t>
-  </si>
-  <si>
     <t>3|0|0</t>
   </si>
   <si>
@@ -110,9 +104,6 @@
     <t>So, why did you join the Force?</t>
   </si>
   <si>
-    <t>Oh, I uh, come from a long line of lawmen-and-women; it was kind of the only thing I could’ve done.|And how long have you been at this job?|I passed Basic Training a couple’a months ago- around the time you left, actually.|Huh- whaddyathink?| I mean, I don’t think it was right of you to leave. You swore the same oath to your brothers and sisters that we all did |*Fuckin’ kid.|I mean about being a cop.|Oh! It’s a good job- gives me the chance to make some real change in this city, and that’s a rare thing.|That it is.</t>
-  </si>
-  <si>
     <t>Happy|Neutral|Neutral|Sad|Angry|Angry|Angry|Neutral|Neutral</t>
   </si>
   <si>
@@ -128,9 +119,6 @@
     <t>What do you think of Sam?</t>
   </si>
   <si>
-    <t> He’s a good man, but his policework- I mean, I don’t want to be rude, but- y’know, he isn’t always the most thorough? Seems to operate more by habit than procedure or anything like that, and it causes oversights- oversights that could get innocent people hurt.|Hm.|*The kid actually cares about the job, Interesting.</t>
-  </si>
-  <si>
     <t>Neutral|Sad|Sad</t>
   </si>
   <si>
@@ -149,7 +137,121 @@
     <t>Sad|Sad|Neutral|Neutral|Sad|Neutral</t>
   </si>
   <si>
-    <t>Oh, yeah- they’re nice, they’re plenty nice… |*His voice trails off- there’s something here.|You sound unsure.|I mean, they’re- they’re their own group, and I’m not saying there’s something wrong with it, but-|but you’re not a part of it. |No, no I'm not.</t>
+    <t>How Sam Treats youu</t>
+  </si>
+  <si>
+    <t>Happy|Neutral|Neutral</t>
+  </si>
+  <si>
+    <t>3|0|3</t>
+  </si>
+  <si>
+    <t>Eoin Richardson|Detective Juels|Eoin Richardson</t>
+  </si>
+  <si>
+    <t>Treatment</t>
+  </si>
+  <si>
+    <t>Add</t>
+  </si>
+  <si>
+    <t>Egt</t>
+  </si>
+  <si>
+    <t>Off Duty?</t>
+  </si>
+  <si>
+    <t>What do you like to do off duty?</t>
+  </si>
+  <si>
+    <t>Neutral|Neutral|Angry|Angry|Happy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time </t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Treatment|Time</t>
+  </si>
+  <si>
+    <t>Add|Add</t>
+  </si>
+  <si>
+    <t>1|1</t>
+  </si>
+  <si>
+    <t>Egt|Egt</t>
+  </si>
+  <si>
+    <t>2|2</t>
+  </si>
+  <si>
+    <t>3|1|0|2|0</t>
+  </si>
+  <si>
+    <t>Eoin Richardson|Detective Juels|Detective Juels|Eoin Richardson|Detective Juels</t>
+  </si>
+  <si>
+    <t>Romance</t>
+  </si>
+  <si>
+    <t>So, are you single? Romantically, I mean.</t>
+  </si>
+  <si>
+    <t>Sad|Angry|Angry|Sad</t>
+  </si>
+  <si>
+    <t>3|1|2|0</t>
+  </si>
+  <si>
+    <t>Eoin Richardson|Detective Juels|Eoin Richardson|Detective Juels</t>
+  </si>
+  <si>
+    <t>Romance2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answer the fucking question, Eoin. </t>
+  </si>
+  <si>
+    <t>Angry|Sad|Sad</t>
+  </si>
+  <si>
+    <t>1|3|3</t>
+  </si>
+  <si>
+    <t>Detective Juels|Eoin Richardson|Eoin Richardson</t>
+  </si>
+  <si>
+    <t>What brings you here? Doesn't really seem like your scene.</t>
+  </si>
+  <si>
+    <t>Uh- well- y'know, the boys were going out, and they ended up inviting me along. I didn't know we were going- to be honest, I assumed we were going to go get dinner down at the diner or something, but- uh- I guess not. I tried to leave, but I saw Sam, and I just… didn't want to leave the guy alone, y'know?|*He stares pointedly at me, the resentment writ large on his face.|I do. Trust me.</t>
+  </si>
+  <si>
+    <t>Oh, I uh, come from a long line of lawmen-and-women; it was kind of the only thing I could've done.|And how long have you been at this job?|I passed Basic Training a couple'a months ago- around the time you left, actually.|Huh- whaddyathink?| I mean, I don't think it was right of you to leave. You swore the same oath to your brothers and sisters that we all did |*Fuckin' kid.|I mean about being a cop.|Oh! It's a good job- gives me the chance to make some real change in this city, and that's a rare thing.|That it is.</t>
+  </si>
+  <si>
+    <t> He's a good man, but his policework- I mean, I don't want to be rude, but- y'know, he isn't always the most thorough? Seems to operate more by habit than procedure or anything like that, and it causes oversights- oversights that could get innocent people hurt.|Hm.|*The kid actually cares about the job, Interesting.</t>
+  </si>
+  <si>
+    <t>Oh, yeah- they're nice, they're plenty nice… |*His voice trails off- there's something here.|You sound unsure.|I mean, they're- they're their own group, and I'm not saying there's something wrong with it, but-|but you're not a part of it. |No, no I'm not.</t>
+  </si>
+  <si>
+    <t> How's Diggums treated you as a partner?</t>
+  </si>
+  <si>
+    <t>Oh- really good. he doesn't care that I'm young, or that I don't drink- he's a good friend. I owe him- I just wish I could help him out somehow.|Maybe there is| Yeah, Maybe</t>
+  </si>
+  <si>
+    <t>Honestly, I haven't had a whole ton of time off- but- uh- I really like adventure novels. Y'know Jordan Steele-the author?|Yeah, I know him.|Thieving Asshole|What was that?|Oh, nothing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kind of a weird question. Why, are you and Sam- |absolutely not. Kid, you gotta learn to stay in your lane with the questions.|I would tell you to do the same thing, Ms. Jefferson. But, from what I've heard, you not doing that's what made you such a darn good detective.|*This kid- why I oughta- wait. He's deflecting- trying to throw me off balance. I should go in for the kill. </t>
+  </si>
+  <si>
+    <t>I know you judge me for leaving the force- for leaving Sam. I get it. but I promise you, I did it for the same reason you joined.|*The fresh-faced officer freezes like a deer illuminated by the muzzle flash of a hunter.|Uh- fine. Sure. I'm single- I mean, I've dated before, but, uh- people usually don't find me-|</t>
   </si>
 </sst>
 </file>
@@ -205,6 +307,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -524,7 +630,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDEE49D1-F89E-464F-BA81-AAC15EF51999}">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.453125" style="1" customWidth="1"/>
@@ -534,7 +640,8 @@
     <col min="5" max="5" width="17.36328125" style="1" customWidth="1"/>
     <col min="6" max="6" width="10.36328125" style="1" customWidth="1"/>
     <col min="7" max="7" width="10.26953125" style="1" customWidth="1"/>
-    <col min="8" max="9" width="8.7265625" style="1"/>
+    <col min="8" max="8" width="12.08984375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="8.7265625" style="1"/>
     <col min="10" max="10" width="21.453125" style="1" customWidth="1"/>
     <col min="11" max="11" width="15.6328125" style="1" customWidth="1"/>
     <col min="12" max="12" width="18.6328125" style="1" customWidth="1"/>
@@ -590,13 +697,13 @@
         <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>14</v>
@@ -608,19 +715,19 @@
         <v>0</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="J2" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M2" s="1">
         <v>0</v>
@@ -631,16 +738,16 @@
     </row>
     <row r="3" spans="1:14" ht="174" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>14</v>
@@ -652,19 +759,19 @@
         <v>0</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J3" s="1">
-        <v>0</v>
+        <v>37</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>46</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="M3" s="1">
         <v>0</v>
@@ -675,16 +782,16 @@
     </row>
     <row r="4" spans="1:14" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>29</v>
+        <v>64</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>14</v>
@@ -696,19 +803,19 @@
         <v>0</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J4" s="1">
-        <v>0</v>
+        <v>45</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>46</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M4" s="1">
         <v>0</v>
@@ -719,16 +826,16 @@
     </row>
     <row r="5" spans="1:14" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>14</v>
@@ -740,25 +847,201 @@
         <v>0</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J5" s="1">
-        <v>0</v>
+        <v>45</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>46</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="M5" s="1">
         <v>0</v>
       </c>
       <c r="N5">
         <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="58" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6" s="1">
+        <v>1</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M6" s="1">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="87" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" s="1">
+        <v>2</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J7" s="1">
+        <v>1</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M7" s="1">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J8" s="1">
+        <v>1</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="M8" s="1">
+        <v>0</v>
+      </c>
+      <c r="N8" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" s="1">
+        <v>0</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="M9" s="1">
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>